<commit_message>
Add actuals comparison and per-project group scoping to the forecast
予測シートに実績を並べ、案件が行わない行程グループを予測から外せるようにした。
あわせて、着手前の案件で分かっているのが要素別の見積もりだけになる将来の
運用に備え、見積もりを正式な入力経路として用意した(設計書 6 Step1 の制約の階層)。

- estimates シート(案件ID / 行程グループ / 見積人月)を追加。任意シートなので
  1行も無ければ従来どおり 契約人月 × 学習比率 で配分する。見積もりがある場合は
  その値をそのままグループ別総量とし、書かれていない行程グループは
  「この案件では行わない業務」として列ごと除外する。契約人月とずれる場合は
  総量として見積もり側を採用し、差を注記に出す(どちらが正かは人が決める)。
- 見積もりがまだ無い段階向けに --exclude-group を追加。総工数は動かさず、
  残ったグループへ学習比率の割合を保ったまま配分し直す。
- 予測シートに 月 × 行程グループ の実績表と、月次の 予測 vs 実績(差分・消化率)
  を追加。実績が無ければその旨だけ出す。列配置を予測表と揃えてあるため、
  合計は数式のままどちらの表からも検算できる。
- 予測対象の案件を学習から除外。進行中の案件は実績が途中までしか無く、
  カーブを合計1に正規化する都合で「前半に全部消化する案件」として学習され、
  平均カーブが前に倒れる。自分自身を学習データにする情報漏れでもある。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EzcNRY8EVx6HeGCEMZT8ER
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="milestones" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase_map" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="projects" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="estimates" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="milestones" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="phase_map" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="settings" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -965,6 +966,49 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>案件ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>行程グループ</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>見積人月</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>【凡例】着手前の案件は実績が無く、要素別の見積もりだけが分かっている。ここに 行程グループ ごとの見積人月を入れると、その値がそのままグループ別の総量になる(設計書 6 Step1)。行を書かなかった行程グループは『この案件では行わない業務』として予測から除外される。1行も無ければ 契約人月 × 学習した工数比率 で配分する。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1614,7 +1658,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2301,7 +2345,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Accept month-level milestone dates and place them at mid-month
マイルストーンを開始・終了と同じ「2020-08」の粒度で書けるようにした。
2020/8 と 2020年8月 も読む。日まで書いた 2020-08-22 とも混在してよい。

月表記はその月の中央として扱う。月初として扱うと、実際の日付が月内に散っている
ぶんだけ全案件のマイルストーンが半月ぶん前へ寄る。同じ向きにずれるので、
案件数を増やしても消えない系統誤差になる。

完了30件で粒度を比べた実測(月次誤差WAPE):

  日まで              0.2898
  月まで(月央として扱う) 0.3008   日との差 +0.011(相対 4%)
  月まで(月末として扱う) 0.3130
  月まで(月初として扱う) 0.3245   日との差 +0.035(相対 12%)

日まで書く効果は小さい。案件ごとに見ると月央のほうが良かった案件が30件中13件あり、
差の95%信頼区間は -0.001〜+0.023 で0をまたぐ(t=1.84)。実績が月単位である以上、
日を細かくするより記入する案件を増やすほうが効く。
一方、月初として扱う実装は日と月の差より大きく悪化するので、月央にする意味は大きい。

セルに 2020-08 と入力すると Excel が 2020-08-01 に変換してしまうことがあり、
そうなると読み込み側では月表記と区別がつかず、月初として扱う状態のまま気づけない。
その受け皿として settings に マイルストーン精度(自動 / 月)を追加した。
月 にすると日付の細部を捨てて月央へ揃える。CLI は --ms-precision 月。
同じ月に入った複数回のマイルストーンがまとまった件数は警告に出す。

settings をマイルストーンの読み込みより前に確定させるよう load_all の順序を入れ替えた。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MkKJ798vbBM96RYupVrfTB
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -1923,7 +1923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2032,95 +2032,112 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>位置合わせ強度</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>1</v>
+          <t>マイルストーン精度</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>自動</t>
+        </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>0〜1。実位置を正準位置へ引き戻す割合。下げると時間軸の伸縮が緩み、工数の跳ねが減る</t>
+          <t>自動 / 月。月 にすると日付を月央に丸める(月まで表記に揃える)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>伸縮率上限</t>
+          <t>位置合わせ強度</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>時間軸の伸縮率の上限(倍)。例 1.5。0=無制限。跳ねの高さに直接上限をかける</t>
+          <t>0〜1。実位置を正準位置へ引き戻す割合。下げると時間軸の伸縮が緩み、工数の跳ねが減る</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>マイルストーン最小件数</t>
+          <t>伸縮率上限</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>この件数未満の統計は参考値として警告する(設計書 11)</t>
+          <t>時間軸の伸縮率の上限(倍)。例 1.5。0=無制限。跳ねの高さに直接上限をかける</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>カーブ解像度</t>
+          <t>マイルストーン最小件数</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>正準時間軸の分割数。学習カーブのビン数</t>
+          <t>この件数未満の統計は参考値として警告する(設計書 11)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>k</t>
+          <t>カーブ解像度</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>種別重み w=n/(n+k)。第1版では未使用。実装順序 3 で使用する</t>
+          <t>正準時間軸の分割数。学習カーブのビン数</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>種別重み w=n/(n+k)。第1版では未使用。実装順序 3 で使用する</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>タグ重み係数</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B13" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>タグ類似度の効き。第1版では未使用。実装順序 4 で使用する</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>【凡例】青字セルが手入力項目。k とタグ重み係数は設計書 9 の実装順序 3・4 で使用予定。第1版(素朴版+位置合わせ)では読み込むだけで計算に使わない。</t>
         </is>

</xml_diff>

<commit_message>
Default milestone dates to month precision
マイルストーン精度 の既定を 自動 から 月 にした。すべてのマイルストーンを
月精度とみなし、月央へ丸める。日の精度をそのまま使いたい場合だけ 自動 にする。

理由は2つ。実績が月単位である以上、日まで書いても得るものが小さいこと
(完了30件で相対4%、95%信頼区間が0をまたぐ)。そして、セルに 2020-08 と入力すると
Excel が 2020-08-01 という日付に変換してしまうことがあり、そうなると読み込み側では
月表記と区別がつかず、月初として扱う状態(相対12%悪化)のまま気づけないこと。
既定が 月 ならこの事故が起きない。

サンプル生成も既定で月表記(2020-08)を書き出すようにし、シートの見た目と
実際に使われる値を一致させた。--date-precision 日 で従来の日表記も出せる。

日まで書かれた日付を丸めたときは件数を警告に出す。既定なので毎回出さず、
実際に細部を捨てたときだけ出す。月に丸めた結果、同じ月に入った複数回の
マイルストーンが1件にまとまった場合も件数を出す。

既定が変わったので README の実測値を月精度で測り直した。結論は変わらない。

  カーブの形ごと(位置合わせ)  後半集中 0.299 / 標準 0.216 / 二山 0.339 / 前倒し 0.399
  やり直しを学習に混ぜる      外す 0.309 -> 使う 0.315   害も益も小さい
  アンカーは最終回            最終回 0.285 / 初回 0.377 / α版を使わない 0.351
  「(初回)」を背骨に入れる     0.273 -> 0.344 と悪化

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MkKJ798vbBM96RYupVrfTB
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -572,22 +572,22 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>2019-10-05</t>
+          <t>2019-10</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>2020-10-17</t>
+          <t>2020-10</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>2021-08-12</t>
+          <t>2021-08</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>2022-01-02</t>
+          <t>2022-01</t>
         </is>
       </c>
     </row>
@@ -635,17 +635,17 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>2020-09-06</t>
+          <t>2020-09</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>2020-11-12</t>
+          <t>2020-11</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>2021-01-28</t>
+          <t>2021-01</t>
         </is>
       </c>
     </row>
@@ -690,22 +690,22 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2021-01-15</t>
+          <t>2021-01</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>2021-09-30</t>
+          <t>2021-09</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>2022-02-10</t>
+          <t>2022-02</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>2022-10-07</t>
+          <t>2022-10</t>
         </is>
       </c>
     </row>
@@ -753,17 +753,17 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>2021-12-19</t>
+          <t>2021-12</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>2022-03-27</t>
+          <t>2022-03</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>2022-05-24</t>
+          <t>2022-05</t>
         </is>
       </c>
     </row>
@@ -808,22 +808,22 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>2021-10-25</t>
+          <t>2021-10</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>2022-04-03</t>
+          <t>2022-04</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>2023-03-07</t>
+          <t>2023-03</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>2023-08-31</t>
+          <t>2023-08</t>
         </is>
       </c>
     </row>
@@ -871,17 +871,17 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>2022-12-09</t>
+          <t>2022-12</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>2023-06-12</t>
+          <t>2023-06</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>2023-08-09</t>
+          <t>2023-08</t>
         </is>
       </c>
     </row>
@@ -926,22 +926,22 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>2022-07-09</t>
+          <t>2022-07</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>2023-01-02</t>
+          <t>2023-01</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>2023-07-25</t>
+          <t>2023-07</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>2023-12-12</t>
+          <t>2023-12</t>
         </is>
       </c>
     </row>
@@ -989,17 +989,17 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>2023-09-23</t>
+          <t>2023-09</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>2024-04-27</t>
+          <t>2024-04</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>2024-07-31</t>
+          <t>2024-07</t>
         </is>
       </c>
     </row>
@@ -1047,17 +1047,17 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>2024-01-27</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>2024-05-01</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>2024-09-23</t>
+          <t>2024-09</t>
         </is>
       </c>
     </row>
@@ -1102,22 +1102,22 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>2025-04-07</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>2025-09-22</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>2027-07-16</t>
+          <t>2027-07</t>
         </is>
       </c>
       <c r="K12" s="3" t="n">
@@ -1178,7 +1178,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>【凡例】青字セルが手入力項目。ステータス=予測対象 の案件が予測の対象になる(実績CSVに行が無くてよい)。ステータス列より右はマイルストーン列で、見出しがマイルストーン名、セルが日付(YYYY-MM-DD)。空欄=未記入で、記入が無くても動作する(設計書 3-2)。同じマイルストーンを一度で通過できず複数回訪れた場合は、同じセルにカンマ区切りで並べる(例: 2020-04-18, 2020-08-22)。列は増やさない。最終回を工程の境目、初回を「α版(初回)」という別のマイルストーンとして扱う。</t>
+          <t>【凡例】青字セルが手入力項目。ステータス=予測対象 の案件が予測の対象になる(実績CSVに行が無くてよい)。ステータス列より右はマイルストーン列で、見出しがマイルストーン名、セルが日付(YYYY-MM-DD)。空欄=未記入で、記入が無くても動作する(設計書 3-2)。同じマイルストーンを一度で通過できず複数回訪れた場合は、同じセルにカンマ区切りで並べる(例: 2020-04, 2020-08)。列は増やさない。最終回を工程の境目、初回を「α版(初回)」という別のマイルストーンとして扱う。</t>
         </is>
       </c>
     </row>
@@ -2037,12 +2037,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>自動</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>自動 / 月。月 にすると日付を月央に丸める(月まで表記に揃える)</t>
+          <t>月 / 自動。既定の 月 は日付を月央に丸める。自動 は日まで書いた日付をそのまま使う</t>
         </is>
       </c>
     </row>

</xml_diff>